<commit_message>
Benchmark: thread a model field through drafts → scorecards → report
The drafting model is part of what a benchmark measures, but it lived only
in the session-log prose. Carry it with the data instead:

- draft meta gains a `model` field (and the draft _TEMPLATE.md slot)
- scorecard template gains a Model header row (relabel row 9 + move Reviewer
  to the blank row 10; no formula/dropdown shift)
- fill_scorecard.py fills the Model row from meta.model
- scorecards_to_csv.py emits a `model` CSV column
- benchmark_report.py treats `model` as a reserved column and auto-derives
  the provenance-footer model from the CSV (--model still overrides)

3 new regression tests; smoke 7/7, 97 tests green.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/07-Standards/curation-benchmarking/PHI-Weaver-Curation-Scorecard.xlsx
+++ b/07-Standards/curation-benchmarking/PHI-Weaver-Curation-Scorecard.xlsx
@@ -171,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -239,6 +239,8 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -634,7 +636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -648,6 +650,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -660,6 +663,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
@@ -672,6 +676,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="90" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
@@ -687,6 +692,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
@@ -699,6 +705,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
@@ -711,6 +718,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="60" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
@@ -723,6 +731,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
@@ -732,6 +741,18 @@
       <c r="B15" s="3" t="inlineStr">
         <is>
           <t>A curation scored all-Correct with full completeness is, by definition, a validated gold-standard example — add it to 07-Standards/curation-examples/.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Model row (header): the LLM/curator that produced the draft, e.g. "Fable 5". Part of what the benchmark measures — keep it constant across a run and record it. fill_scorecard.py fills it from the draft; scorecards_to_csv.py carries it into the report provenance.</t>
         </is>
       </c>
     </row>
@@ -781,10 +802,10 @@
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr"/>
-      <c r="C4" s="7" t="n"/>
-      <c r="D4" s="7" t="n"/>
-      <c r="E4" s="7" t="n"/>
-      <c r="F4" s="7" t="n"/>
+      <c r="C4" s="27" t="n"/>
+      <c r="D4" s="27" t="n"/>
+      <c r="E4" s="27" t="n"/>
+      <c r="F4" s="28" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -793,10 +814,10 @@
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr"/>
-      <c r="C5" s="7" t="n"/>
-      <c r="D5" s="7" t="n"/>
-      <c r="E5" s="7" t="n"/>
-      <c r="F5" s="7" t="n"/>
+      <c r="C5" s="27" t="n"/>
+      <c r="D5" s="27" t="n"/>
+      <c r="E5" s="27" t="n"/>
+      <c r="F5" s="28" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -805,10 +826,10 @@
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="7" t="n"/>
-      <c r="D6" s="7" t="n"/>
-      <c r="E6" s="7" t="n"/>
-      <c r="F6" s="7" t="n"/>
+      <c r="C6" s="27" t="n"/>
+      <c r="D6" s="27" t="n"/>
+      <c r="E6" s="27" t="n"/>
+      <c r="F6" s="28" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -817,10 +838,10 @@
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
-      <c r="F7" s="7" t="n"/>
+      <c r="C7" s="27" t="n"/>
+      <c r="D7" s="27" t="n"/>
+      <c r="E7" s="27" t="n"/>
+      <c r="F7" s="28" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -829,22 +850,34 @@
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr"/>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="n"/>
-      <c r="F8" s="7" t="n"/>
+      <c r="C8" s="27" t="n"/>
+      <c r="D8" s="27" t="n"/>
+      <c r="E8" s="27" t="n"/>
+      <c r="F8" s="28" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr"/>
+      <c r="C9" s="27" t="n"/>
+      <c r="D9" s="27" t="n"/>
+      <c r="E9" s="27" t="n"/>
+      <c r="F9" s="28" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
           <t>Reviewer (2nd curator)</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="7" t="n"/>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="27" t="n"/>
+      <c r="D10" s="27" t="n"/>
+      <c r="E10" s="27" t="n"/>
+      <c r="F10" s="28" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
@@ -1216,8 +1249,8 @@
           <t>Completeness</t>
         </is>
       </c>
-      <c r="B30" s="19" t="n"/>
-      <c r="C30" s="19" t="n"/>
+      <c r="B30" s="27" t="n"/>
+      <c r="C30" s="28" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -1225,7 +1258,7 @@
           <t>Curatable items in the paper</t>
         </is>
       </c>
-      <c r="B31" s="20" t="n"/>
+      <c r="B31" s="28" t="n"/>
       <c r="C31" s="12" t="n">
         <v>0</v>
       </c>
@@ -1236,7 +1269,7 @@
           <t>Items captured in the draft</t>
         </is>
       </c>
-      <c r="B32" s="20" t="n"/>
+      <c r="B32" s="28" t="n"/>
       <c r="C32" s="12" t="n">
         <v>0</v>
       </c>
@@ -1247,7 +1280,7 @@
           <t>Items missed</t>
         </is>
       </c>
-      <c r="B33" s="20" t="n"/>
+      <c r="B33" s="28" t="n"/>
       <c r="C33" s="12">
         <f>MAX(0,C31-C32)</f>
         <v/>
@@ -1259,20 +1292,21 @@
           <t>Completeness</t>
         </is>
       </c>
-      <c r="B34" s="20" t="n"/>
+      <c r="B34" s="28" t="n"/>
       <c r="C34" s="21">
         <f>IF(C31=0,"",C32/C31)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="A33:B33"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B10:F10"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="A32:B32"/>
     <mergeCell ref="A30:C30"/>

</xml_diff>

<commit_message>
Scorecard: drop "(incl. effector GO:0140418)" from the GO item label
The GO / gene annotation item is a general scoring row; the effector-GO
parenthetical was over-specific (not every paper has an effector, and the
effector-GO rule now lives in the gene-for-gene skill). Fixed in both the
generator (make_scorecard.py) and the baked template cell B14. The label
still contains "go / gene annotation", so fill_scorecard.py's substring
matcher is unaffected (verified: GO row still prefills, formula intact).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/07-Standards/curation-benchmarking/PHI-Weaver-Curation-Scorecard.xlsx
+++ b/07-Standards/curation-benchmarking/PHI-Weaver-Curation-Scorecard.xlsx
@@ -650,7 +650,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -663,7 +662,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
@@ -676,7 +674,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="90" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
@@ -692,7 +689,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
@@ -705,7 +701,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
@@ -718,7 +713,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="60" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
@@ -731,7 +725,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
@@ -965,7 +958,7 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>GO / gene annotation correctness (incl. effector GO:0140418)</t>
+          <t>GO / gene annotation correctness</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">

</xml_diff>